<commit_message>
Update Suggestions v2 with corrected property URLs
</commit_message>
<xml_diff>
--- a/Suggestions v2.xlsx
+++ b/Suggestions v2.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E9687647-9A75-43C1-812C-03BE7A609B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD1D92E3-F00F-499B-BF9B-B02338042B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -251,9 +251,6 @@
     <t>2550</t>
   </si>
   <si>
-    <t>https://www.qterrapropertymanagement.com/properties/28-200-malta-ave%2C-brampton%2C-ontario%2C-l6y-6h8</t>
-  </si>
-  <si>
     <t>28-200 Malta Ave, Brampton, Ontario L6Y 6H8</t>
   </si>
   <si>
@@ -818,9 +815,6 @@
     <t>267-60 Parrotta Dr, Toronto, Ontario M9M 0E5</t>
   </si>
   <si>
-    <t>https://www.qterrapropertymanagement.com/properties/3-823-stirling-ave-s%2C-kitchener%2C-ontario%2C-n2m-3k4</t>
-  </si>
-  <si>
     <t>3-823 Stirling Ave S, Kitchener, Ontario N2M 3K4</t>
   </si>
   <si>
@@ -1235,9 +1229,6 @@
     <t>2-208 Clarence St., Ottawa, Ontario K1N 5R1</t>
   </si>
   <si>
-    <t>https://www.qterrapropertymanagement.com/properties/2-56-garthdale-ct%2C-toronto%2C-ontario-m3h-5p9</t>
-  </si>
-  <si>
     <t>1-56 Garthdale Ct, Toronto, Ontario M3H 5P9</t>
   </si>
   <si>
@@ -1367,9 +1358,6 @@
     <t>3-232 Lawrence Ave W, Toronto, Ontario M4R 2J3</t>
   </si>
   <si>
-    <t>https://www.qterrapropertymanagement.com/properties/5364-glen-erin-dr%2C-mississauga%2C-ontario-l5m-5c2</t>
-  </si>
-  <si>
     <t>5364 Glen Erin Dr, Mississauga, Ontario L5M 5C2</t>
   </si>
   <si>
@@ -1590,16 +1578,36 @@
   </si>
   <si>
     <t>Price</t>
+  </si>
+  <si>
+    <t>https://www.qterrapropertymanagement.com/properties/28-200-malta-ave%2C-brampton%2C-ontario-l6y-6h8</t>
+  </si>
+  <si>
+    <t>https://www.qterrapropertymanagement.com/properties/3-823-stirling-ave-s%2C-kitchener%2C-ontario-n2m-3k4</t>
+  </si>
+  <si>
+    <t>https://www.qterrapropertymanagement.com/properties/1-56-garthdale-ct%2C-toronto%2C-ontario-m3h-5p9</t>
+  </si>
+  <si>
+    <t>https://www.qterrapropertymanagement.com/properties/5364-gerin-dr%2C-mississauga%2C-ontario-l5m-5c2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1613,7 +1621,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1621,14 +1629,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1976,25 +2004,25 @@
     <col min="5" max="5" width="33.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1" t="s">
+        <v>517</v>
+      </c>
+      <c r="C1" t="s">
+        <v>518</v>
+      </c>
+      <c r="D1" t="s">
+        <v>519</v>
+      </c>
+      <c r="E1" t="s">
         <v>520</v>
       </c>
-      <c r="B1" t="s">
-        <v>521</v>
-      </c>
-      <c r="C1" t="s">
-        <v>522</v>
-      </c>
-      <c r="D1" t="s">
-        <v>523</v>
-      </c>
-      <c r="E1" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    </row>
+    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
@@ -2010,8 +2038,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B3" t="s">
@@ -2027,8 +2055,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B4" t="s">
@@ -2044,8 +2072,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B5" t="s">
@@ -2061,8 +2089,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B6" t="s">
@@ -2078,8 +2106,8 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B7" t="s">
@@ -2095,8 +2123,8 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B8" t="s">
@@ -2112,8 +2140,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B9" t="s">
@@ -2129,8 +2157,8 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B10" t="s">
@@ -2146,8 +2174,8 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B11" t="s">
@@ -2163,8 +2191,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B12" t="s">
@@ -2180,8 +2208,8 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B13" t="s">
@@ -2197,8 +2225,8 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B14" t="s">
@@ -2214,8 +2242,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
         <v>45</v>
       </c>
       <c r="B15" t="s">
@@ -2231,8 +2259,8 @@
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="16" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
         <v>49</v>
       </c>
       <c r="B16" t="s">
@@ -2248,8 +2276,8 @@
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B17" t="s">
@@ -2265,8 +2293,8 @@
         <v>54</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="18" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
         <v>55</v>
       </c>
       <c r="B18" t="s">
@@ -2282,8 +2310,8 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B19" t="s">
@@ -2299,8 +2327,8 @@
         <v>60</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B20" t="s">
@@ -2316,8 +2344,8 @@
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="21" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B21" t="s">
@@ -2333,8 +2361,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="22" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B22" t="s">
@@ -2350,8 +2378,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="23" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B23" t="s">
@@ -2367,8 +2395,8 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="24" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
         <v>70</v>
       </c>
       <c r="B24" t="s">
@@ -2384,8 +2412,8 @@
         <v>72</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="25" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
         <v>73</v>
       </c>
       <c r="B25" t="s">
@@ -2401,8 +2429,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="26" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
         <v>75</v>
       </c>
       <c r="B26" t="s">
@@ -2418,12 +2446,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="27" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="B27" t="s">
         <v>78</v>
-      </c>
-      <c r="B27" t="s">
-        <v>79</v>
       </c>
       <c r="C27" t="s">
         <v>2</v>
@@ -2435,12 +2463,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="28" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B28" t="s">
         <v>80</v>
-      </c>
-      <c r="B28" t="s">
-        <v>81</v>
       </c>
       <c r="C28" t="s">
         <v>2</v>
@@ -2449,32 +2477,32 @@
         <v>22</v>
       </c>
       <c r="E28" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="B29" t="s">
         <v>83</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
+        <v>2</v>
+      </c>
+      <c r="D29" t="s">
         <v>84</v>
-      </c>
-      <c r="C29" t="s">
-        <v>2</v>
-      </c>
-      <c r="D29" t="s">
-        <v>85</v>
       </c>
       <c r="E29" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="30" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B30" t="s">
         <v>86</v>
-      </c>
-      <c r="B30" t="s">
-        <v>87</v>
       </c>
       <c r="C30" t="s">
         <v>2</v>
@@ -2483,15 +2511,15 @@
         <v>18</v>
       </c>
       <c r="E30" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="B31" t="s">
         <v>89</v>
-      </c>
-      <c r="B31" t="s">
-        <v>90</v>
       </c>
       <c r="C31" t="s">
         <v>2</v>
@@ -2500,15 +2528,15 @@
         <v>18</v>
       </c>
       <c r="E31" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="B32" t="s">
         <v>92</v>
-      </c>
-      <c r="B32" t="s">
-        <v>93</v>
       </c>
       <c r="C32" t="s">
         <v>2</v>
@@ -2517,15 +2545,15 @@
         <v>3</v>
       </c>
       <c r="E32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+      <c r="B33" t="s">
         <v>95</v>
-      </c>
-      <c r="B33" t="s">
-        <v>96</v>
       </c>
       <c r="C33" t="s">
         <v>2</v>
@@ -2534,15 +2562,15 @@
         <v>59</v>
       </c>
       <c r="E33" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+      <c r="B34" t="s">
         <v>98</v>
-      </c>
-      <c r="B34" t="s">
-        <v>99</v>
       </c>
       <c r="C34" t="s">
         <v>2</v>
@@ -2551,15 +2579,15 @@
         <v>3</v>
       </c>
       <c r="E34" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+      <c r="B35" t="s">
         <v>101</v>
-      </c>
-      <c r="B35" t="s">
-        <v>102</v>
       </c>
       <c r="C35" t="s">
         <v>2</v>
@@ -2568,15 +2596,15 @@
         <v>47</v>
       </c>
       <c r="E35" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+      <c r="B36" t="s">
         <v>104</v>
-      </c>
-      <c r="B36" t="s">
-        <v>105</v>
       </c>
       <c r="C36" t="s">
         <v>2</v>
@@ -2585,15 +2613,15 @@
         <v>47</v>
       </c>
       <c r="E36" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B37" t="s">
         <v>106</v>
-      </c>
-      <c r="B37" t="s">
-        <v>107</v>
       </c>
       <c r="C37" t="s">
         <v>2</v>
@@ -2602,32 +2630,32 @@
         <v>34</v>
       </c>
       <c r="E37" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B38" t="s">
         <v>108</v>
       </c>
-      <c r="B38" t="s">
+      <c r="C38" t="s">
+        <v>2</v>
+      </c>
+      <c r="D38" t="s">
         <v>109</v>
-      </c>
-      <c r="C38" t="s">
-        <v>2</v>
-      </c>
-      <c r="D38" t="s">
-        <v>110</v>
       </c>
       <c r="E38" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="39" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B39" t="s">
         <v>111</v>
-      </c>
-      <c r="B39" t="s">
-        <v>112</v>
       </c>
       <c r="C39" t="s">
         <v>2</v>
@@ -2636,15 +2664,15 @@
         <v>59</v>
       </c>
       <c r="E39" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B40" t="s">
         <v>113</v>
-      </c>
-      <c r="B40" t="s">
-        <v>114</v>
       </c>
       <c r="C40" t="s">
         <v>2</v>
@@ -2656,12 +2684,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+    <row r="41" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B41" t="s">
         <v>115</v>
-      </c>
-      <c r="B41" t="s">
-        <v>116</v>
       </c>
       <c r="C41" t="s">
         <v>2</v>
@@ -2670,15 +2698,15 @@
         <v>34</v>
       </c>
       <c r="E41" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B42" t="s">
         <v>117</v>
-      </c>
-      <c r="B42" t="s">
-        <v>118</v>
       </c>
       <c r="C42" t="s">
         <v>2</v>
@@ -2690,12 +2718,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+    <row r="43" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B43" t="s">
         <v>119</v>
-      </c>
-      <c r="B43" t="s">
-        <v>120</v>
       </c>
       <c r="C43" t="s">
         <v>2</v>
@@ -2704,15 +2732,15 @@
         <v>34</v>
       </c>
       <c r="E43" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+      <c r="B44" t="s">
         <v>122</v>
-      </c>
-      <c r="B44" t="s">
-        <v>123</v>
       </c>
       <c r="C44" t="s">
         <v>2</v>
@@ -2724,12 +2752,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+    <row r="45" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B45" t="s">
         <v>124</v>
-      </c>
-      <c r="B45" t="s">
-        <v>125</v>
       </c>
       <c r="C45" t="s">
         <v>2</v>
@@ -2738,15 +2766,15 @@
         <v>67</v>
       </c>
       <c r="E45" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+      <c r="B46" t="s">
         <v>127</v>
-      </c>
-      <c r="B46" t="s">
-        <v>128</v>
       </c>
       <c r="C46" t="s">
         <v>14</v>
@@ -2758,12 +2786,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+    <row r="47" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B47" t="s">
         <v>129</v>
-      </c>
-      <c r="B47" t="s">
-        <v>130</v>
       </c>
       <c r="C47" t="s">
         <v>2</v>
@@ -2772,15 +2800,15 @@
         <v>22</v>
       </c>
       <c r="E47" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
+      <c r="B48" t="s">
         <v>132</v>
-      </c>
-      <c r="B48" t="s">
-        <v>133</v>
       </c>
       <c r="C48" t="s">
         <v>2</v>
@@ -2789,15 +2817,15 @@
         <v>18</v>
       </c>
       <c r="E48" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B49" t="s">
         <v>134</v>
-      </c>
-      <c r="B49" t="s">
-        <v>135</v>
       </c>
       <c r="C49" t="s">
         <v>14</v>
@@ -2806,15 +2834,15 @@
         <v>22</v>
       </c>
       <c r="E49" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B50" t="s">
         <v>136</v>
-      </c>
-      <c r="B50" t="s">
-        <v>137</v>
       </c>
       <c r="C50" t="s">
         <v>14</v>
@@ -2823,15 +2851,15 @@
         <v>3</v>
       </c>
       <c r="E50" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+      <c r="B51" t="s">
         <v>139</v>
-      </c>
-      <c r="B51" t="s">
-        <v>140</v>
       </c>
       <c r="C51" t="s">
         <v>2</v>
@@ -2840,15 +2868,15 @@
         <v>18</v>
       </c>
       <c r="E51" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="1" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+      <c r="B52" t="s">
         <v>142</v>
-      </c>
-      <c r="B52" t="s">
-        <v>143</v>
       </c>
       <c r="C52" t="s">
         <v>2</v>
@@ -2857,15 +2885,15 @@
         <v>34</v>
       </c>
       <c r="E52" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B53" t="s">
         <v>144</v>
-      </c>
-      <c r="B53" t="s">
-        <v>145</v>
       </c>
       <c r="C53" t="s">
         <v>2</v>
@@ -2877,12 +2905,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
+    <row r="54" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B54" t="s">
         <v>146</v>
-      </c>
-      <c r="B54" t="s">
-        <v>147</v>
       </c>
       <c r="C54" t="s">
         <v>2</v>
@@ -2891,15 +2919,15 @@
         <v>47</v>
       </c>
       <c r="E54" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="1" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+      <c r="B55" t="s">
         <v>149</v>
-      </c>
-      <c r="B55" t="s">
-        <v>150</v>
       </c>
       <c r="C55" t="s">
         <v>2</v>
@@ -2908,49 +2936,49 @@
         <v>3</v>
       </c>
       <c r="E55" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
+      <c r="B56" t="s">
         <v>152</v>
-      </c>
-      <c r="B56" t="s">
-        <v>153</v>
       </c>
       <c r="C56" t="s">
         <v>14</v>
       </c>
       <c r="D56" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E56" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B57" t="s">
         <v>154</v>
       </c>
-      <c r="B57" t="s">
+      <c r="C57" t="s">
+        <v>2</v>
+      </c>
+      <c r="D57" t="s">
         <v>155</v>
-      </c>
-      <c r="C57" t="s">
-        <v>2</v>
-      </c>
-      <c r="D57" t="s">
-        <v>156</v>
       </c>
       <c r="E57" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+    <row r="58" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B58" t="s">
         <v>157</v>
-      </c>
-      <c r="B58" t="s">
-        <v>158</v>
       </c>
       <c r="C58" t="s">
         <v>2</v>
@@ -2959,15 +2987,15 @@
         <v>18</v>
       </c>
       <c r="E58" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B59" t="s">
         <v>159</v>
-      </c>
-      <c r="B59" t="s">
-        <v>160</v>
       </c>
       <c r="C59" t="s">
         <v>2</v>
@@ -2976,15 +3004,15 @@
         <v>47</v>
       </c>
       <c r="E59" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="1" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+      <c r="B60" t="s">
         <v>162</v>
-      </c>
-      <c r="B60" t="s">
-        <v>163</v>
       </c>
       <c r="C60" t="s">
         <v>2</v>
@@ -2993,15 +3021,15 @@
         <v>59</v>
       </c>
       <c r="E60" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="1" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+      <c r="B61" t="s">
         <v>165</v>
-      </c>
-      <c r="B61" t="s">
-        <v>166</v>
       </c>
       <c r="C61" t="s">
         <v>14</v>
@@ -3010,15 +3038,15 @@
         <v>18</v>
       </c>
       <c r="E61" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="1" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+      <c r="B62" t="s">
         <v>168</v>
-      </c>
-      <c r="B62" t="s">
-        <v>169</v>
       </c>
       <c r="C62" t="s">
         <v>2</v>
@@ -3027,15 +3055,15 @@
         <v>34</v>
       </c>
       <c r="E62" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B63" t="s">
         <v>170</v>
-      </c>
-      <c r="B63" t="s">
-        <v>171</v>
       </c>
       <c r="C63" t="s">
         <v>2</v>
@@ -3044,15 +3072,15 @@
         <v>18</v>
       </c>
       <c r="E63" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="1" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
+      <c r="B64" t="s">
         <v>173</v>
-      </c>
-      <c r="B64" t="s">
-        <v>174</v>
       </c>
       <c r="C64" t="s">
         <v>2</v>
@@ -3061,15 +3089,15 @@
         <v>67</v>
       </c>
       <c r="E64" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="1" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
+      <c r="B65" t="s">
         <v>176</v>
-      </c>
-      <c r="B65" t="s">
-        <v>177</v>
       </c>
       <c r="C65" t="s">
         <v>2</v>
@@ -3078,15 +3106,15 @@
         <v>47</v>
       </c>
       <c r="E65" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B66" t="s">
         <v>178</v>
-      </c>
-      <c r="B66" t="s">
-        <v>179</v>
       </c>
       <c r="C66" t="s">
         <v>2</v>
@@ -3095,15 +3123,15 @@
         <v>3</v>
       </c>
       <c r="E66" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B67" t="s">
         <v>180</v>
-      </c>
-      <c r="B67" t="s">
-        <v>181</v>
       </c>
       <c r="C67" t="s">
         <v>2</v>
@@ -3112,32 +3140,32 @@
         <v>18</v>
       </c>
       <c r="E67" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B68" t="s">
         <v>182</v>
       </c>
-      <c r="B68" t="s">
+      <c r="C68" t="s">
+        <v>2</v>
+      </c>
+      <c r="D68" t="s">
+        <v>109</v>
+      </c>
+      <c r="E68" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="C68" t="s">
-        <v>2</v>
-      </c>
-      <c r="D68" t="s">
-        <v>110</v>
-      </c>
-      <c r="E68" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+      <c r="B69" t="s">
         <v>184</v>
-      </c>
-      <c r="B69" t="s">
-        <v>185</v>
       </c>
       <c r="C69" t="s">
         <v>2</v>
@@ -3146,15 +3174,15 @@
         <v>34</v>
       </c>
       <c r="E69" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B70" t="s">
         <v>186</v>
-      </c>
-      <c r="B70" t="s">
-        <v>187</v>
       </c>
       <c r="C70" t="s">
         <v>2</v>
@@ -3166,12 +3194,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+    <row r="71" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="B71" t="s">
         <v>188</v>
-      </c>
-      <c r="B71" t="s">
-        <v>189</v>
       </c>
       <c r="C71" t="s">
         <v>2</v>
@@ -3180,15 +3208,15 @@
         <v>47</v>
       </c>
       <c r="E71" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="1" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+      <c r="B72" t="s">
         <v>191</v>
-      </c>
-      <c r="B72" t="s">
-        <v>192</v>
       </c>
       <c r="C72" t="s">
         <v>2</v>
@@ -3197,15 +3225,15 @@
         <v>18</v>
       </c>
       <c r="E72" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B73" t="s">
         <v>193</v>
-      </c>
-      <c r="B73" t="s">
-        <v>194</v>
       </c>
       <c r="C73" t="s">
         <v>2</v>
@@ -3214,15 +3242,15 @@
         <v>18</v>
       </c>
       <c r="E73" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="B74" t="s">
         <v>195</v>
-      </c>
-      <c r="B74" t="s">
-        <v>196</v>
       </c>
       <c r="C74" t="s">
         <v>2</v>
@@ -3231,15 +3259,15 @@
         <v>18</v>
       </c>
       <c r="E74" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="B75" t="s">
         <v>197</v>
-      </c>
-      <c r="B75" t="s">
-        <v>198</v>
       </c>
       <c r="C75" t="s">
         <v>2</v>
@@ -3248,15 +3276,15 @@
         <v>3</v>
       </c>
       <c r="E75" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="B76" t="s">
         <v>199</v>
-      </c>
-      <c r="B76" t="s">
-        <v>200</v>
       </c>
       <c r="C76" t="s">
         <v>2</v>
@@ -3268,12 +3296,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+    <row r="77" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B77" t="s">
         <v>201</v>
-      </c>
-      <c r="B77" t="s">
-        <v>202</v>
       </c>
       <c r="C77" t="s">
         <v>2</v>
@@ -3285,12 +3313,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
+    <row r="78" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B78" t="s">
         <v>203</v>
-      </c>
-      <c r="B78" t="s">
-        <v>204</v>
       </c>
       <c r="C78" t="s">
         <v>2</v>
@@ -3299,15 +3327,15 @@
         <v>18</v>
       </c>
       <c r="E78" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="1" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
+      <c r="B79" t="s">
         <v>206</v>
-      </c>
-      <c r="B79" t="s">
-        <v>207</v>
       </c>
       <c r="C79" t="s">
         <v>2</v>
@@ -3316,15 +3344,15 @@
         <v>34</v>
       </c>
       <c r="E79" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="B80" t="s">
         <v>208</v>
-      </c>
-      <c r="B80" t="s">
-        <v>209</v>
       </c>
       <c r="C80" t="s">
         <v>14</v>
@@ -3333,32 +3361,32 @@
         <v>47</v>
       </c>
       <c r="E80" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="1" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
+      <c r="B81" t="s">
         <v>211</v>
       </c>
-      <c r="B81" t="s">
-        <v>212</v>
-      </c>
       <c r="C81" t="s">
         <v>2</v>
       </c>
       <c r="D81" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E81" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
+    <row r="82" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="B82" t="s">
         <v>213</v>
-      </c>
-      <c r="B82" t="s">
-        <v>214</v>
       </c>
       <c r="C82" t="s">
         <v>2</v>
@@ -3367,15 +3395,15 @@
         <v>67</v>
       </c>
       <c r="E82" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="B83" t="s">
         <v>215</v>
-      </c>
-      <c r="B83" t="s">
-        <v>216</v>
       </c>
       <c r="C83" t="s">
         <v>2</v>
@@ -3384,15 +3412,15 @@
         <v>47</v>
       </c>
       <c r="E83" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B84" t="s">
         <v>217</v>
-      </c>
-      <c r="B84" t="s">
-        <v>218</v>
       </c>
       <c r="C84" t="s">
         <v>2</v>
@@ -3401,15 +3429,15 @@
         <v>3</v>
       </c>
       <c r="E84" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="1" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
+      <c r="B85" t="s">
         <v>220</v>
-      </c>
-      <c r="B85" t="s">
-        <v>221</v>
       </c>
       <c r="C85" t="s">
         <v>2</v>
@@ -3421,12 +3449,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
+    <row r="86" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B86" t="s">
         <v>222</v>
-      </c>
-      <c r="B86" t="s">
-        <v>223</v>
       </c>
       <c r="C86" t="s">
         <v>2</v>
@@ -3435,15 +3463,15 @@
         <v>3</v>
       </c>
       <c r="E86" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="1" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
+      <c r="B87" t="s">
         <v>225</v>
-      </c>
-      <c r="B87" t="s">
-        <v>226</v>
       </c>
       <c r="C87" t="s">
         <v>2</v>
@@ -3455,12 +3483,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
+    <row r="88" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="B88" t="s">
         <v>227</v>
-      </c>
-      <c r="B88" t="s">
-        <v>228</v>
       </c>
       <c r="C88" t="s">
         <v>2</v>
@@ -3469,15 +3497,15 @@
         <v>7</v>
       </c>
       <c r="E88" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="1" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
+      <c r="B89" t="s">
         <v>230</v>
-      </c>
-      <c r="B89" t="s">
-        <v>231</v>
       </c>
       <c r="C89" t="s">
         <v>2</v>
@@ -3486,15 +3514,15 @@
         <v>18</v>
       </c>
       <c r="E89" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="B90" t="s">
         <v>232</v>
-      </c>
-      <c r="B90" t="s">
-        <v>233</v>
       </c>
       <c r="C90" t="s">
         <v>2</v>
@@ -3506,12 +3534,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
+    <row r="91" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="B91" t="s">
         <v>234</v>
-      </c>
-      <c r="B91" t="s">
-        <v>235</v>
       </c>
       <c r="C91" t="s">
         <v>2</v>
@@ -3520,15 +3548,15 @@
         <v>47</v>
       </c>
       <c r="E91" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="1" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
+      <c r="B92" t="s">
         <v>237</v>
-      </c>
-      <c r="B92" t="s">
-        <v>238</v>
       </c>
       <c r="C92" t="s">
         <v>14</v>
@@ -3537,32 +3565,32 @@
         <v>34</v>
       </c>
       <c r="E92" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="B93" t="s">
         <v>239</v>
       </c>
-      <c r="B93" t="s">
+      <c r="C93" t="s">
+        <v>2</v>
+      </c>
+      <c r="D93" t="s">
+        <v>84</v>
+      </c>
+      <c r="E93" t="s">
         <v>240</v>
       </c>
-      <c r="C93" t="s">
-        <v>2</v>
-      </c>
-      <c r="D93" t="s">
-        <v>85</v>
-      </c>
-      <c r="E93" t="s">
+    </row>
+    <row r="94" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="1" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
+      <c r="B94" t="s">
         <v>242</v>
-      </c>
-      <c r="B94" t="s">
-        <v>243</v>
       </c>
       <c r="C94" t="s">
         <v>2</v>
@@ -3571,15 +3599,15 @@
         <v>47</v>
       </c>
       <c r="E94" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="1" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
+      <c r="B95" t="s">
         <v>245</v>
-      </c>
-      <c r="B95" t="s">
-        <v>246</v>
       </c>
       <c r="C95" t="s">
         <v>2</v>
@@ -3591,12 +3619,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
+    <row r="96" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="B96" t="s">
         <v>247</v>
-      </c>
-      <c r="B96" t="s">
-        <v>248</v>
       </c>
       <c r="C96" t="s">
         <v>2</v>
@@ -3605,15 +3633,15 @@
         <v>22</v>
       </c>
       <c r="E96" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="1" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
+      <c r="B97" t="s">
         <v>250</v>
-      </c>
-      <c r="B97" t="s">
-        <v>251</v>
       </c>
       <c r="C97" t="s">
         <v>2</v>
@@ -3622,15 +3650,15 @@
         <v>18</v>
       </c>
       <c r="E97" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="B98" t="s">
         <v>252</v>
-      </c>
-      <c r="B98" t="s">
-        <v>253</v>
       </c>
       <c r="C98" t="s">
         <v>2</v>
@@ -3642,12 +3670,12 @@
         <v>51</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
+    <row r="99" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="B99" t="s">
         <v>254</v>
-      </c>
-      <c r="B99" t="s">
-        <v>255</v>
       </c>
       <c r="C99" t="s">
         <v>2</v>
@@ -3659,12 +3687,12 @@
         <v>51</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
+    <row r="100" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="B100" t="s">
         <v>256</v>
-      </c>
-      <c r="B100" t="s">
-        <v>257</v>
       </c>
       <c r="C100" t="s">
         <v>2</v>
@@ -3673,15 +3701,15 @@
         <v>3</v>
       </c>
       <c r="E100" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B101" t="s">
         <v>258</v>
-      </c>
-      <c r="B101" t="s">
-        <v>259</v>
       </c>
       <c r="C101" t="s">
         <v>2</v>
@@ -3693,12 +3721,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
+    <row r="102" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B102" t="s">
         <v>260</v>
-      </c>
-      <c r="B102" t="s">
-        <v>261</v>
       </c>
       <c r="C102" t="s">
         <v>14</v>
@@ -3707,32 +3735,32 @@
         <v>3</v>
       </c>
       <c r="E102" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="1" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
+      <c r="B103" t="s">
         <v>263</v>
       </c>
-      <c r="B103" t="s">
-        <v>264</v>
-      </c>
       <c r="C103" t="s">
         <v>2</v>
       </c>
       <c r="D103" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E103" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
+    <row r="104" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="B104" t="s">
         <v>265</v>
-      </c>
-      <c r="B104" t="s">
-        <v>266</v>
       </c>
       <c r="C104" t="s">
         <v>2</v>
@@ -3741,15 +3769,15 @@
         <v>67</v>
       </c>
       <c r="E104" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
-        <v>267</v>
+        <v>163</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A105" s="1" t="s">
+        <v>522</v>
       </c>
       <c r="B105" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C105" t="s">
         <v>2</v>
@@ -3758,15 +3786,15 @@
         <v>59</v>
       </c>
       <c r="E105" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
-        <v>269</v>
+        <v>261</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A106" s="1" t="s">
+        <v>267</v>
       </c>
       <c r="B106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C106" t="s">
         <v>2</v>
@@ -3778,63 +3806,63 @@
         <v>77</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
+    <row r="107" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A107" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="B107" t="s">
+        <v>270</v>
+      </c>
+      <c r="C107" t="s">
+        <v>2</v>
+      </c>
+      <c r="D107" t="s">
+        <v>84</v>
+      </c>
+      <c r="E107" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A108" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B108" t="s">
         <v>272</v>
       </c>
-      <c r="C107" t="s">
-        <v>2</v>
-      </c>
-      <c r="D107" t="s">
-        <v>85</v>
-      </c>
-      <c r="E107" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
+      <c r="C108" t="s">
+        <v>2</v>
+      </c>
+      <c r="D108" t="s">
+        <v>109</v>
+      </c>
+      <c r="E108" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A109" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B109" t="s">
         <v>274</v>
       </c>
-      <c r="C108" t="s">
-        <v>2</v>
-      </c>
-      <c r="D108" t="s">
-        <v>110</v>
-      </c>
-      <c r="E108" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
+      <c r="C109" t="s">
+        <v>2</v>
+      </c>
+      <c r="D109" t="s">
+        <v>109</v>
+      </c>
+      <c r="E109" t="s">
         <v>275</v>
       </c>
-      <c r="B109" t="s">
+    </row>
+    <row r="110" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A110" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="C109" t="s">
-        <v>2</v>
-      </c>
-      <c r="D109" t="s">
-        <v>110</v>
-      </c>
-      <c r="E109" t="s">
+      <c r="B110" t="s">
         <v>277</v>
-      </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>278</v>
-      </c>
-      <c r="B110" t="s">
-        <v>279</v>
       </c>
       <c r="C110" t="s">
         <v>14</v>
@@ -3843,32 +3871,32 @@
         <v>59</v>
       </c>
       <c r="E110" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A111" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="B111" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
+      <c r="C111" t="s">
+        <v>2</v>
+      </c>
+      <c r="D111" t="s">
+        <v>109</v>
+      </c>
+      <c r="E111" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A112" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="B111" t="s">
+      <c r="B112" t="s">
         <v>282</v>
-      </c>
-      <c r="C111" t="s">
-        <v>2</v>
-      </c>
-      <c r="D111" t="s">
-        <v>110</v>
-      </c>
-      <c r="E111" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
-        <v>283</v>
-      </c>
-      <c r="B112" t="s">
-        <v>284</v>
       </c>
       <c r="C112" t="s">
         <v>2</v>
@@ -3877,15 +3905,15 @@
         <v>18</v>
       </c>
       <c r="E112" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A113" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B113" t="s">
         <v>285</v>
-      </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
-        <v>286</v>
-      </c>
-      <c r="B113" t="s">
-        <v>287</v>
       </c>
       <c r="C113" t="s">
         <v>14</v>
@@ -3897,12 +3925,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
-        <v>288</v>
+    <row r="114" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A114" s="1" t="s">
+        <v>286</v>
       </c>
       <c r="B114" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C114" t="s">
         <v>2</v>
@@ -3914,29 +3942,29 @@
         <v>77</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>290</v>
+    <row r="115" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A115" s="1" t="s">
+        <v>288</v>
       </c>
       <c r="B115" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C115" t="s">
         <v>2</v>
       </c>
       <c r="D115" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E115" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
-        <v>292</v>
+    <row r="116" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A116" s="1" t="s">
+        <v>290</v>
       </c>
       <c r="B116" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C116" t="s">
         <v>14</v>
@@ -3945,32 +3973,32 @@
         <v>59</v>
       </c>
       <c r="E116" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>294</v>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A117" s="1" t="s">
+        <v>292</v>
       </c>
       <c r="B117" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C117" t="s">
         <v>2</v>
       </c>
       <c r="D117" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E117" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>296</v>
+    <row r="118" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A118" s="1" t="s">
+        <v>294</v>
       </c>
       <c r="B118" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C118" t="s">
         <v>14</v>
@@ -3979,15 +4007,15 @@
         <v>18</v>
       </c>
       <c r="E118" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>298</v>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A119" s="1" t="s">
+        <v>296</v>
       </c>
       <c r="B119" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C119" t="s">
         <v>14</v>
@@ -3999,12 +4027,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
-        <v>300</v>
+    <row r="120" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A120" s="1" t="s">
+        <v>298</v>
       </c>
       <c r="B120" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C120" t="s">
         <v>2</v>
@@ -4013,15 +4041,15 @@
         <v>18</v>
       </c>
       <c r="E120" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>302</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A121" s="1" t="s">
+        <v>300</v>
       </c>
       <c r="B121" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C121" t="s">
         <v>14</v>
@@ -4030,15 +4058,15 @@
         <v>67</v>
       </c>
       <c r="E121" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A122" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="B122" t="s">
         <v>304</v>
-      </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
-        <v>305</v>
-      </c>
-      <c r="B122" t="s">
-        <v>306</v>
       </c>
       <c r="C122" t="s">
         <v>2</v>
@@ -4047,15 +4075,15 @@
         <v>18</v>
       </c>
       <c r="E122" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A123" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="B123" t="s">
         <v>307</v>
-      </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
-        <v>308</v>
-      </c>
-      <c r="B123" t="s">
-        <v>309</v>
       </c>
       <c r="C123" t="s">
         <v>2</v>
@@ -4064,15 +4092,15 @@
         <v>47</v>
       </c>
       <c r="E123" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A124" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="B124" t="s">
         <v>310</v>
-      </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
-        <v>311</v>
-      </c>
-      <c r="B124" t="s">
-        <v>312</v>
       </c>
       <c r="C124" t="s">
         <v>2</v>
@@ -4084,29 +4112,29 @@
         <v>41</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
-        <v>313</v>
+    <row r="125" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A125" s="1" t="s">
+        <v>311</v>
       </c>
       <c r="B125" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C125" t="s">
         <v>14</v>
       </c>
       <c r="D125" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E125" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A126" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="B126" t="s">
         <v>315</v>
-      </c>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
-        <v>316</v>
-      </c>
-      <c r="B126" t="s">
-        <v>317</v>
       </c>
       <c r="C126" t="s">
         <v>14</v>
@@ -4115,15 +4143,15 @@
         <v>47</v>
       </c>
       <c r="E126" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A127" t="s">
-        <v>318</v>
+        <v>209</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A127" s="1" t="s">
+        <v>316</v>
       </c>
       <c r="B127" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C127" t="s">
         <v>2</v>
@@ -4135,12 +4163,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
-        <v>320</v>
+    <row r="128" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A128" s="1" t="s">
+        <v>318</v>
       </c>
       <c r="B128" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C128" t="s">
         <v>2</v>
@@ -4149,32 +4177,32 @@
         <v>3</v>
       </c>
       <c r="E128" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A129" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="B129" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A129" t="s">
+      <c r="C129" t="s">
+        <v>2</v>
+      </c>
+      <c r="D129" t="s">
+        <v>109</v>
+      </c>
+      <c r="E129" t="s">
         <v>323</v>
       </c>
-      <c r="B129" t="s">
+    </row>
+    <row r="130" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A130" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="C129" t="s">
-        <v>2</v>
-      </c>
-      <c r="D129" t="s">
-        <v>110</v>
-      </c>
-      <c r="E129" t="s">
+      <c r="B130" t="s">
         <v>325</v>
-      </c>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A130" t="s">
-        <v>326</v>
-      </c>
-      <c r="B130" t="s">
-        <v>327</v>
       </c>
       <c r="C130" t="s">
         <v>2</v>
@@ -4183,15 +4211,15 @@
         <v>67</v>
       </c>
       <c r="E130" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A131" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="B131" t="s">
         <v>328</v>
-      </c>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A131" t="s">
-        <v>329</v>
-      </c>
-      <c r="B131" t="s">
-        <v>330</v>
       </c>
       <c r="C131" t="s">
         <v>2</v>
@@ -4203,12 +4231,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A132" t="s">
-        <v>331</v>
+    <row r="132" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A132" s="1" t="s">
+        <v>329</v>
       </c>
       <c r="B132" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="C132" t="s">
         <v>2</v>
@@ -4217,15 +4245,15 @@
         <v>18</v>
       </c>
       <c r="E132" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A133" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="B133" t="s">
         <v>333</v>
-      </c>
-    </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A133" t="s">
-        <v>334</v>
-      </c>
-      <c r="B133" t="s">
-        <v>335</v>
       </c>
       <c r="C133" t="s">
         <v>2</v>
@@ -4237,12 +4265,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A134" t="s">
-        <v>336</v>
+    <row r="134" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A134" s="1" t="s">
+        <v>334</v>
       </c>
       <c r="B134" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C134" t="s">
         <v>2</v>
@@ -4254,12 +4282,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A135" t="s">
-        <v>338</v>
+    <row r="135" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A135" s="1" t="s">
+        <v>336</v>
       </c>
       <c r="B135" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C135" t="s">
         <v>2</v>
@@ -4268,15 +4296,15 @@
         <v>18</v>
       </c>
       <c r="E135" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A136" t="s">
-        <v>340</v>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A136" s="1" t="s">
+        <v>338</v>
       </c>
       <c r="B136" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C136" t="s">
         <v>2</v>
@@ -4285,15 +4313,15 @@
         <v>22</v>
       </c>
       <c r="E136" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A137" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="B137" t="s">
         <v>342</v>
-      </c>
-    </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A137" t="s">
-        <v>343</v>
-      </c>
-      <c r="B137" t="s">
-        <v>344</v>
       </c>
       <c r="C137" t="s">
         <v>2</v>
@@ -4305,12 +4333,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A138" t="s">
-        <v>345</v>
+    <row r="138" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A138" s="1" t="s">
+        <v>343</v>
       </c>
       <c r="B138" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C138" t="s">
         <v>2</v>
@@ -4322,12 +4350,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A139" t="s">
-        <v>347</v>
+    <row r="139" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A139" s="1" t="s">
+        <v>345</v>
       </c>
       <c r="B139" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C139" t="s">
         <v>14</v>
@@ -4339,12 +4367,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A140" t="s">
-        <v>349</v>
+    <row r="140" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A140" s="1" t="s">
+        <v>347</v>
       </c>
       <c r="B140" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C140" t="s">
         <v>14</v>
@@ -4356,12 +4384,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A141" t="s">
-        <v>351</v>
+    <row r="141" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A141" s="1" t="s">
+        <v>349</v>
       </c>
       <c r="B141" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C141" t="s">
         <v>2</v>
@@ -4370,15 +4398,15 @@
         <v>34</v>
       </c>
       <c r="E141" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A142" t="s">
-        <v>353</v>
+        <v>305</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A142" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="B142" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C142" t="s">
         <v>14</v>
@@ -4387,15 +4415,15 @@
         <v>22</v>
       </c>
       <c r="E142" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A143" t="s">
-        <v>355</v>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A143" s="1" t="s">
+        <v>353</v>
       </c>
       <c r="B143" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C143" t="s">
         <v>2</v>
@@ -4404,15 +4432,15 @@
         <v>3</v>
       </c>
       <c r="E143" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A144" t="s">
-        <v>357</v>
+        <v>261</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A144" s="1" t="s">
+        <v>355</v>
       </c>
       <c r="B144" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C144" t="s">
         <v>14</v>
@@ -4424,12 +4452,12 @@
         <v>23</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A145" t="s">
-        <v>359</v>
+    <row r="145" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A145" s="1" t="s">
+        <v>357</v>
       </c>
       <c r="B145" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C145" t="s">
         <v>2</v>
@@ -4438,15 +4466,15 @@
         <v>47</v>
       </c>
       <c r="E145" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A146" t="s">
-        <v>361</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A146" s="1" t="s">
+        <v>359</v>
       </c>
       <c r="B146" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C146" t="s">
         <v>2</v>
@@ -4458,12 +4486,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A147" t="s">
-        <v>363</v>
+    <row r="147" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A147" s="1" t="s">
+        <v>361</v>
       </c>
       <c r="B147" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C147" t="s">
         <v>14</v>
@@ -4472,32 +4500,32 @@
         <v>18</v>
       </c>
       <c r="E147" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A148" t="s">
-        <v>365</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A148" s="1" t="s">
+        <v>363</v>
       </c>
       <c r="B148" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C148" t="s">
         <v>14</v>
       </c>
       <c r="D148" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E148" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A149" t="s">
-        <v>367</v>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A149" s="1" t="s">
+        <v>365</v>
       </c>
       <c r="B149" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C149" t="s">
         <v>2</v>
@@ -4506,15 +4534,15 @@
         <v>34</v>
       </c>
       <c r="E149" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A150" t="s">
-        <v>369</v>
+        <v>340</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A150" s="1" t="s">
+        <v>367</v>
       </c>
       <c r="B150" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C150" t="s">
         <v>2</v>
@@ -4526,29 +4554,29 @@
         <v>44</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A151" t="s">
-        <v>371</v>
+    <row r="151" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A151" s="1" t="s">
+        <v>369</v>
       </c>
       <c r="B151" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C151" t="s">
         <v>2</v>
       </c>
       <c r="D151" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E151" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A152" t="s">
-        <v>373</v>
+    <row r="152" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A152" s="1" t="s">
+        <v>371</v>
       </c>
       <c r="B152" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C152" t="s">
         <v>14</v>
@@ -4560,12 +4588,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A153" t="s">
-        <v>375</v>
+    <row r="153" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A153" s="1" t="s">
+        <v>373</v>
       </c>
       <c r="B153" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C153" t="s">
         <v>14</v>
@@ -4577,29 +4605,29 @@
         <v>28</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A154" t="s">
+    <row r="154" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A154" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="B154" t="s">
+        <v>376</v>
+      </c>
+      <c r="C154" t="s">
+        <v>2</v>
+      </c>
+      <c r="D154" t="s">
+        <v>155</v>
+      </c>
+      <c r="E154" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A155" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="B154" t="s">
+      <c r="B155" t="s">
         <v>378</v>
-      </c>
-      <c r="C154" t="s">
-        <v>2</v>
-      </c>
-      <c r="D154" t="s">
-        <v>156</v>
-      </c>
-      <c r="E154" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A155" t="s">
-        <v>379</v>
-      </c>
-      <c r="B155" t="s">
-        <v>380</v>
       </c>
       <c r="C155" t="s">
         <v>2</v>
@@ -4608,15 +4636,15 @@
         <v>3</v>
       </c>
       <c r="E155" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A156" t="s">
-        <v>381</v>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A156" s="1" t="s">
+        <v>379</v>
       </c>
       <c r="B156" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C156" t="s">
         <v>2</v>
@@ -4628,12 +4656,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A157" t="s">
-        <v>383</v>
+    <row r="157" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A157" s="1" t="s">
+        <v>381</v>
       </c>
       <c r="B157" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C157" t="s">
         <v>2</v>
@@ -4642,15 +4670,15 @@
         <v>34</v>
       </c>
       <c r="E157" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A158" t="s">
-        <v>385</v>
+        <v>340</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A158" s="1" t="s">
+        <v>383</v>
       </c>
       <c r="B158" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C158" t="s">
         <v>14</v>
@@ -4659,15 +4687,15 @@
         <v>18</v>
       </c>
       <c r="E158" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A159" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="B159" t="s">
         <v>387</v>
-      </c>
-    </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A159" t="s">
-        <v>388</v>
-      </c>
-      <c r="B159" t="s">
-        <v>389</v>
       </c>
       <c r="C159" t="s">
         <v>2</v>
@@ -4676,32 +4704,32 @@
         <v>3</v>
       </c>
       <c r="E159" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A160" t="s">
-        <v>390</v>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A160" s="1" t="s">
+        <v>388</v>
       </c>
       <c r="B160" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C160" t="s">
         <v>2</v>
       </c>
       <c r="D160" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E160" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A161" t="s">
-        <v>392</v>
+    <row r="161" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A161" s="1" t="s">
+        <v>390</v>
       </c>
       <c r="B161" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="C161" t="s">
         <v>2</v>
@@ -4710,15 +4738,15 @@
         <v>3</v>
       </c>
       <c r="E161" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A162" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="B162" t="s">
         <v>394</v>
-      </c>
-    </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A162" t="s">
-        <v>395</v>
-      </c>
-      <c r="B162" t="s">
-        <v>396</v>
       </c>
       <c r="C162" t="s">
         <v>14</v>
@@ -4727,15 +4755,15 @@
         <v>18</v>
       </c>
       <c r="E162" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A163" t="s">
-        <v>397</v>
+        <v>171</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A163" s="1" t="s">
+        <v>395</v>
       </c>
       <c r="B163" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="C163" t="s">
         <v>2</v>
@@ -4747,29 +4775,29 @@
         <v>44</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A164" t="s">
+    <row r="164" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A164" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="B164" t="s">
+        <v>398</v>
+      </c>
+      <c r="C164" t="s">
+        <v>2</v>
+      </c>
+      <c r="D164" t="s">
+        <v>84</v>
+      </c>
+      <c r="E164" t="s">
         <v>399</v>
       </c>
-      <c r="B164" t="s">
+    </row>
+    <row r="165" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A165" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="C164" t="s">
-        <v>2</v>
-      </c>
-      <c r="D164" t="s">
-        <v>85</v>
-      </c>
-      <c r="E164" t="s">
+      <c r="B165" t="s">
         <v>401</v>
-      </c>
-    </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A165" t="s">
-        <v>402</v>
-      </c>
-      <c r="B165" t="s">
-        <v>403</v>
       </c>
       <c r="C165" t="s">
         <v>14</v>
@@ -4781,29 +4809,29 @@
         <v>44</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A166" t="s">
-        <v>404</v>
+    <row r="166" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A166" s="1" t="s">
+        <v>402</v>
       </c>
       <c r="B166" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C166" t="s">
         <v>2</v>
       </c>
       <c r="D166" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E166" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A167" t="s">
-        <v>406</v>
+    <row r="167" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A167" s="1" t="s">
+        <v>523</v>
       </c>
       <c r="B167" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="C167" t="s">
         <v>2</v>
@@ -4815,12 +4843,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A168" t="s">
-        <v>408</v>
+    <row r="168" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A168" s="1" t="s">
+        <v>405</v>
       </c>
       <c r="B168" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="C168" t="s">
         <v>14</v>
@@ -4829,15 +4857,15 @@
         <v>3</v>
       </c>
       <c r="E168" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A169" t="s">
-        <v>410</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A169" s="1" t="s">
+        <v>407</v>
       </c>
       <c r="B169" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="C169" t="s">
         <v>14</v>
@@ -4849,12 +4877,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A170" t="s">
-        <v>412</v>
+    <row r="170" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A170" s="1" t="s">
+        <v>409</v>
       </c>
       <c r="B170" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="C170" t="s">
         <v>2</v>
@@ -4863,15 +4891,15 @@
         <v>7</v>
       </c>
       <c r="E170" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A171" t="s">
-        <v>415</v>
+        <v>411</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A171" s="1" t="s">
+        <v>412</v>
       </c>
       <c r="B171" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="C171" t="s">
         <v>2</v>
@@ -4883,12 +4911,12 @@
         <v>51</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A172" t="s">
-        <v>417</v>
+    <row r="172" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A172" s="1" t="s">
+        <v>414</v>
       </c>
       <c r="B172" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="C172" t="s">
         <v>2</v>
@@ -4900,12 +4928,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A173" t="s">
-        <v>419</v>
+    <row r="173" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A173" s="1" t="s">
+        <v>416</v>
       </c>
       <c r="B173" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="C173" t="s">
         <v>14</v>
@@ -4914,15 +4942,15 @@
         <v>34</v>
       </c>
       <c r="E173" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A174" t="s">
-        <v>421</v>
+        <v>137</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A174" s="1" t="s">
+        <v>418</v>
       </c>
       <c r="B174" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="C174" t="s">
         <v>14</v>
@@ -4931,15 +4959,15 @@
         <v>18</v>
       </c>
       <c r="E174" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A175" t="s">
-        <v>423</v>
+        <v>171</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A175" s="1" t="s">
+        <v>420</v>
       </c>
       <c r="B175" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="C175" t="s">
         <v>14</v>
@@ -4951,12 +4979,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A176" t="s">
-        <v>425</v>
+    <row r="176" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A176" s="1" t="s">
+        <v>422</v>
       </c>
       <c r="B176" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="C176" t="s">
         <v>14</v>
@@ -4968,29 +4996,29 @@
         <v>72</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A177" t="s">
+    <row r="177" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A177" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="B177" t="s">
+        <v>425</v>
+      </c>
+      <c r="C177" t="s">
+        <v>2</v>
+      </c>
+      <c r="D177" t="s">
+        <v>84</v>
+      </c>
+      <c r="E177" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A178" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="B177" t="s">
+      <c r="B178" t="s">
         <v>428</v>
-      </c>
-      <c r="C177" t="s">
-        <v>2</v>
-      </c>
-      <c r="D177" t="s">
-        <v>85</v>
-      </c>
-      <c r="E177" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A178" t="s">
-        <v>430</v>
-      </c>
-      <c r="B178" t="s">
-        <v>431</v>
       </c>
       <c r="C178" t="s">
         <v>2</v>
@@ -5002,12 +5030,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A179" t="s">
-        <v>432</v>
+    <row r="179" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A179" s="1" t="s">
+        <v>429</v>
       </c>
       <c r="B179" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="C179" t="s">
         <v>14</v>
@@ -5019,12 +5047,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A180" t="s">
-        <v>434</v>
+    <row r="180" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A180" s="1" t="s">
+        <v>431</v>
       </c>
       <c r="B180" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="C180" t="s">
         <v>14</v>
@@ -5033,15 +5061,15 @@
         <v>18</v>
       </c>
       <c r="E180" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A181" t="s">
-        <v>436</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A181" s="1" t="s">
+        <v>433</v>
       </c>
       <c r="B181" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="C181" t="s">
         <v>14</v>
@@ -5050,15 +5078,15 @@
         <v>3</v>
       </c>
       <c r="E181" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A182" t="s">
-        <v>439</v>
+        <v>435</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A182" s="1" t="s">
+        <v>436</v>
       </c>
       <c r="B182" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="C182" t="s">
         <v>14</v>
@@ -5067,15 +5095,15 @@
         <v>22</v>
       </c>
       <c r="E182" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A183" t="s">
-        <v>441</v>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A183" s="1" t="s">
+        <v>438</v>
       </c>
       <c r="B183" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="C183" t="s">
         <v>2</v>
@@ -5084,32 +5112,32 @@
         <v>34</v>
       </c>
       <c r="E183" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A184" t="s">
-        <v>443</v>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A184" s="1" t="s">
+        <v>440</v>
       </c>
       <c r="B184" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="C184" t="s">
         <v>2</v>
       </c>
       <c r="D184" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E184" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A185" t="s">
-        <v>445</v>
+    <row r="185" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A185" s="1" t="s">
+        <v>442</v>
       </c>
       <c r="B185" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="C185" t="s">
         <v>14</v>
@@ -5118,32 +5146,32 @@
         <v>18</v>
       </c>
       <c r="E185" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A186" t="s">
-        <v>448</v>
+        <v>444</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A186" s="1" t="s">
+        <v>445</v>
       </c>
       <c r="B186" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="C186" t="s">
         <v>2</v>
       </c>
       <c r="D186" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E186" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A187" t="s">
-        <v>450</v>
+    <row r="187" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A187" s="1" t="s">
+        <v>524</v>
       </c>
       <c r="B187" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="C187" t="s">
         <v>2</v>
@@ -5152,32 +5180,32 @@
         <v>22</v>
       </c>
       <c r="E187" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A188" t="s">
-        <v>453</v>
+        <v>448</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A188" s="1" t="s">
+        <v>449</v>
       </c>
       <c r="B188" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="C188" t="s">
         <v>2</v>
       </c>
       <c r="D188" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E188" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A189" t="s">
-        <v>455</v>
+    <row r="189" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A189" s="1" t="s">
+        <v>451</v>
       </c>
       <c r="B189" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="C189" t="s">
         <v>2</v>
@@ -5186,32 +5214,32 @@
         <v>22</v>
       </c>
       <c r="E189" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A190" t="s">
-        <v>458</v>
+        <v>453</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A190" s="1" t="s">
+        <v>454</v>
       </c>
       <c r="B190" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="C190" t="s">
         <v>2</v>
       </c>
       <c r="D190" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E190" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A191" t="s">
-        <v>460</v>
+    <row r="191" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A191" s="1" t="s">
+        <v>456</v>
       </c>
       <c r="B191" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="C191" t="s">
         <v>14</v>
@@ -5223,12 +5251,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A192" t="s">
-        <v>462</v>
+    <row r="192" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A192" s="1" t="s">
+        <v>458</v>
       </c>
       <c r="B192" t="s">
-        <v>463</v>
+        <v>459</v>
       </c>
       <c r="C192" t="s">
         <v>2</v>
@@ -5240,29 +5268,29 @@
         <v>28</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A193" t="s">
-        <v>464</v>
+    <row r="193" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A193" s="1" t="s">
+        <v>460</v>
       </c>
       <c r="B193" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="C193" t="s">
         <v>14</v>
       </c>
       <c r="D193" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E193" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A194" t="s">
-        <v>466</v>
+        <v>223</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A194" s="1" t="s">
+        <v>462</v>
       </c>
       <c r="B194" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="C194" t="s">
         <v>14</v>
@@ -5271,49 +5299,49 @@
         <v>3</v>
       </c>
       <c r="E194" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A195" t="s">
-        <v>468</v>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A195" s="1" t="s">
+        <v>464</v>
       </c>
       <c r="B195" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="C195" t="s">
         <v>14</v>
       </c>
       <c r="D195" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E195" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A196" t="s">
-        <v>470</v>
+        <v>275</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A196" s="1" t="s">
+        <v>466</v>
       </c>
       <c r="B196" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="C196" t="s">
         <v>14</v>
       </c>
       <c r="D196" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E196" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A197" t="s">
-        <v>472</v>
+    <row r="197" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A197" s="1" t="s">
+        <v>468</v>
       </c>
       <c r="B197" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="C197" t="s">
         <v>14</v>
@@ -5325,12 +5353,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A198" t="s">
-        <v>474</v>
+    <row r="198" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A198" s="1" t="s">
+        <v>470</v>
       </c>
       <c r="B198" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="C198" t="s">
         <v>14</v>
@@ -5339,15 +5367,15 @@
         <v>18</v>
       </c>
       <c r="E198" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A199" t="s">
-        <v>476</v>
+        <v>171</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A199" s="1" t="s">
+        <v>472</v>
       </c>
       <c r="B199" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
       <c r="C199" t="s">
         <v>14</v>
@@ -5356,15 +5384,15 @@
         <v>67</v>
       </c>
       <c r="E199" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A200" t="s">
-        <v>479</v>
+        <v>474</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A200" s="1" t="s">
+        <v>475</v>
       </c>
       <c r="B200" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="C200" t="s">
         <v>14</v>
@@ -5376,12 +5404,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A201" t="s">
-        <v>481</v>
+    <row r="201" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A201" s="1" t="s">
+        <v>477</v>
       </c>
       <c r="B201" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="C201" t="s">
         <v>14</v>
@@ -5393,12 +5421,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A202" t="s">
-        <v>483</v>
+    <row r="202" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A202" s="1" t="s">
+        <v>479</v>
       </c>
       <c r="B202" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="C202" t="s">
         <v>14</v>
@@ -5410,12 +5438,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A203" t="s">
-        <v>485</v>
+    <row r="203" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A203" s="1" t="s">
+        <v>481</v>
       </c>
       <c r="B203" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="C203" t="s">
         <v>14</v>
@@ -5424,15 +5452,15 @@
         <v>3</v>
       </c>
       <c r="E203" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A204" t="s">
-        <v>487</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A204" s="1" t="s">
+        <v>483</v>
       </c>
       <c r="B204" t="s">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="C204" t="s">
         <v>2</v>
@@ -5441,15 +5469,15 @@
         <v>34</v>
       </c>
       <c r="E204" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A205" t="s">
-        <v>490</v>
+        <v>485</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A205" s="1" t="s">
+        <v>486</v>
       </c>
       <c r="B205" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="C205" t="s">
         <v>2</v>
@@ -5458,15 +5486,15 @@
         <v>3</v>
       </c>
       <c r="E205" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A206" t="s">
-        <v>492</v>
+        <v>426</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A206" s="1" t="s">
+        <v>488</v>
       </c>
       <c r="B206" t="s">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="C206" t="s">
         <v>2</v>
@@ -5475,15 +5503,15 @@
         <v>18</v>
       </c>
       <c r="E206" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A207" t="s">
-        <v>494</v>
+        <v>171</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A207" s="1" t="s">
+        <v>490</v>
       </c>
       <c r="B207" t="s">
-        <v>495</v>
+        <v>491</v>
       </c>
       <c r="C207" t="s">
         <v>2</v>
@@ -5492,15 +5520,15 @@
         <v>47</v>
       </c>
       <c r="E207" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A208" t="s">
-        <v>496</v>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A208" s="1" t="s">
+        <v>492</v>
       </c>
       <c r="B208" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="C208" t="s">
         <v>14</v>
@@ -5509,15 +5537,15 @@
         <v>59</v>
       </c>
       <c r="E208" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A209" t="s">
-        <v>498</v>
+        <v>453</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A209" s="1" t="s">
+        <v>494</v>
       </c>
       <c r="B209" t="s">
-        <v>499</v>
+        <v>495</v>
       </c>
       <c r="C209" t="s">
         <v>2</v>
@@ -5526,15 +5554,15 @@
         <v>22</v>
       </c>
       <c r="E209" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A210" t="s">
-        <v>501</v>
+        <v>496</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A210" s="1" t="s">
+        <v>497</v>
       </c>
       <c r="B210" t="s">
-        <v>502</v>
+        <v>498</v>
       </c>
       <c r="C210" t="s">
         <v>14</v>
@@ -5543,15 +5571,15 @@
         <v>67</v>
       </c>
       <c r="E210" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A211" t="s">
-        <v>504</v>
+        <v>499</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A211" s="1" t="s">
+        <v>500</v>
       </c>
       <c r="B211" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="C211" t="s">
         <v>14</v>
@@ -5560,15 +5588,15 @@
         <v>34</v>
       </c>
       <c r="E211" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A212" t="s">
-        <v>507</v>
+        <v>502</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A212" s="1" t="s">
+        <v>503</v>
       </c>
       <c r="B212" t="s">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="C212" t="s">
         <v>2</v>
@@ -5577,15 +5605,15 @@
         <v>3</v>
       </c>
       <c r="E212" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A213" t="s">
-        <v>510</v>
+        <v>505</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A213" s="1" t="s">
+        <v>506</v>
       </c>
       <c r="B213" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
       <c r="C213" t="s">
         <v>14</v>
@@ -5597,12 +5625,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A214" t="s">
-        <v>512</v>
+    <row r="214" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A214" s="1" t="s">
+        <v>508</v>
       </c>
       <c r="B214" t="s">
-        <v>513</v>
+        <v>509</v>
       </c>
       <c r="C214" t="s">
         <v>14</v>
@@ -5611,32 +5639,32 @@
         <v>34</v>
       </c>
       <c r="E214" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A215" t="s">
-        <v>514</v>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A215" s="1" t="s">
+        <v>510</v>
       </c>
       <c r="B215" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="C215" t="s">
         <v>14</v>
       </c>
       <c r="D215" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E215" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A216" t="s">
-        <v>516</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A216" s="1" t="s">
+        <v>512</v>
       </c>
       <c r="B216" t="s">
-        <v>517</v>
+        <v>513</v>
       </c>
       <c r="C216" t="s">
         <v>14</v>
@@ -5648,12 +5676,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A217" t="s">
-        <v>518</v>
+    <row r="217" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A217" s="1" t="s">
+        <v>514</v>
       </c>
       <c r="B217" t="s">
-        <v>519</v>
+        <v>515</v>
       </c>
       <c r="C217" t="s">
         <v>14</v>
@@ -5666,6 +5694,224 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{CCD8C0F9-F83B-4FCC-863F-04C8497722F7}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{036DB7BB-CA13-46C1-B847-ADEFC88285C7}"/>
+    <hyperlink ref="A4" r:id="rId3" xr:uid="{F1F00EAA-3DEB-4CE2-9C0A-B734650F2A4A}"/>
+    <hyperlink ref="A5" r:id="rId4" xr:uid="{E06C4DC4-8263-48DD-8673-ABED6430898B}"/>
+    <hyperlink ref="A6" r:id="rId5" xr:uid="{07A99E7E-6778-4FED-A9FB-0672F760CCBC}"/>
+    <hyperlink ref="A7" r:id="rId6" xr:uid="{C3C5EE10-E747-4EA5-87A6-5399B4014C6F}"/>
+    <hyperlink ref="A8" r:id="rId7" xr:uid="{641287EA-E94A-4791-9980-7BD3E3D487B7}"/>
+    <hyperlink ref="A9" r:id="rId8" xr:uid="{220A0B6B-62BF-448B-ACC8-5A2B49BC1305}"/>
+    <hyperlink ref="A10" r:id="rId9" xr:uid="{A9B3CDF5-E422-4A43-A975-48E918BFF92C}"/>
+    <hyperlink ref="A11" r:id="rId10" xr:uid="{9B6FC1FB-796A-4669-8D1E-D574087E92B3}"/>
+    <hyperlink ref="A12" r:id="rId11" xr:uid="{56D8BDB4-2164-4CF1-902F-4A4EBF31B4BF}"/>
+    <hyperlink ref="A13" r:id="rId12" xr:uid="{0D3737E9-9716-484D-BA09-71080DAC947C}"/>
+    <hyperlink ref="A14" r:id="rId13" xr:uid="{8DFC04F3-318F-44D0-B18C-511889A9EE05}"/>
+    <hyperlink ref="A15" r:id="rId14" xr:uid="{EE739630-12CC-4466-BF52-82D4366404FA}"/>
+    <hyperlink ref="A16" r:id="rId15" xr:uid="{7AFDC7BE-2C65-4707-8BD6-8D03B8635D1F}"/>
+    <hyperlink ref="A17" r:id="rId16" xr:uid="{09AC5D1A-A89A-422B-A71E-EC25EC5C12E9}"/>
+    <hyperlink ref="A18" r:id="rId17" xr:uid="{55698DF6-0545-41A8-8455-E17B1329F231}"/>
+    <hyperlink ref="A19" r:id="rId18" xr:uid="{F135A30A-AF9E-4171-B7AB-594350AEA823}"/>
+    <hyperlink ref="A20" r:id="rId19" xr:uid="{484B905B-D88F-4A3C-907E-4D9F90F9DBA7}"/>
+    <hyperlink ref="A21" r:id="rId20" xr:uid="{1643B56F-5112-4F21-82B9-87065E137709}"/>
+    <hyperlink ref="A22" r:id="rId21" xr:uid="{60AFDF6F-137F-4813-B275-626AB47B26FE}"/>
+    <hyperlink ref="A23" r:id="rId22" xr:uid="{3A40B990-B898-4F73-B6C4-8F1888BEA484}"/>
+    <hyperlink ref="A24" r:id="rId23" xr:uid="{1C528C55-EDAF-47EE-A964-828380F1E010}"/>
+    <hyperlink ref="A25" r:id="rId24" xr:uid="{FE118020-37C4-405A-AE97-6EA536483693}"/>
+    <hyperlink ref="A26" r:id="rId25" xr:uid="{11256938-2DA1-47D2-846C-AB73083E422F}"/>
+    <hyperlink ref="A27" r:id="rId26" xr:uid="{826314CA-FC92-480A-8A71-7823B1D3499A}"/>
+    <hyperlink ref="A28" r:id="rId27" xr:uid="{5D4DC871-F3D8-410D-8869-938CE8FC8D11}"/>
+    <hyperlink ref="A29" r:id="rId28" xr:uid="{10A0F5D3-35DC-4661-B172-1C778625127B}"/>
+    <hyperlink ref="A30" r:id="rId29" xr:uid="{B56F9696-5D6A-4EDF-A196-B00A3431E033}"/>
+    <hyperlink ref="A31" r:id="rId30" xr:uid="{1B7599FC-210F-450F-9E70-787FC89F42A3}"/>
+    <hyperlink ref="A32" r:id="rId31" xr:uid="{8D6BA266-ADEF-4B59-946C-3CFCD06FADF4}"/>
+    <hyperlink ref="A33" r:id="rId32" xr:uid="{46A31C93-01CA-428E-A34C-F9A671C1D42C}"/>
+    <hyperlink ref="A34" r:id="rId33" xr:uid="{A8B8EA02-660B-4262-BAA0-6C23F72D6968}"/>
+    <hyperlink ref="A35" r:id="rId34" xr:uid="{6EFE2FD3-BD3F-45F5-9218-DFE2946D1099}"/>
+    <hyperlink ref="A36" r:id="rId35" xr:uid="{95C34906-DDB0-4FD2-8C9F-1F4B86596D14}"/>
+    <hyperlink ref="A37" r:id="rId36" xr:uid="{399D0810-A973-48C0-9239-2151B3423EB7}"/>
+    <hyperlink ref="A38" r:id="rId37" xr:uid="{DF7FA386-C810-4AD8-B210-AD99A34AC960}"/>
+    <hyperlink ref="A39" r:id="rId38" xr:uid="{F77DCAE9-A6F0-4F4E-982B-A71F472C0642}"/>
+    <hyperlink ref="A40" r:id="rId39" xr:uid="{9CE345B4-1126-4CB0-AFA0-7FA4EF0B496C}"/>
+    <hyperlink ref="A41" r:id="rId40" xr:uid="{97CAD4BC-F44C-4054-A8B4-F392D81D90E5}"/>
+    <hyperlink ref="A42" r:id="rId41" xr:uid="{7CACBF7C-49ED-4AB6-BE54-DF3DE83520EA}"/>
+    <hyperlink ref="A43" r:id="rId42" xr:uid="{A72C16CC-D858-466A-A8F8-80764D1BAF72}"/>
+    <hyperlink ref="A44" r:id="rId43" xr:uid="{904D0D31-A65C-4775-A2EB-1585968C7C21}"/>
+    <hyperlink ref="A45" r:id="rId44" xr:uid="{E1BA6D05-2BE6-40C1-9A9E-4C6A2537768B}"/>
+    <hyperlink ref="A46" r:id="rId45" xr:uid="{FF5F5317-CE36-4EDD-8B75-288F79039629}"/>
+    <hyperlink ref="A47" r:id="rId46" xr:uid="{9C9CE4AC-9A76-4357-AD37-BFF2EF8D3CA5}"/>
+    <hyperlink ref="A48" r:id="rId47" xr:uid="{9D5BF738-9B14-4303-886F-4B54FA698C98}"/>
+    <hyperlink ref="A49" r:id="rId48" xr:uid="{DC972C2E-754B-47CB-8885-3B5F6BA2BCBA}"/>
+    <hyperlink ref="A50" r:id="rId49" xr:uid="{1C7EB7E0-498A-4540-92D4-C874DC62F896}"/>
+    <hyperlink ref="A51" r:id="rId50" xr:uid="{B34DA1A3-80D7-405B-9914-A81BC237197B}"/>
+    <hyperlink ref="A52" r:id="rId51" xr:uid="{8168E8E8-AAAE-4763-B8E6-C2AFF3A5F411}"/>
+    <hyperlink ref="A53" r:id="rId52" xr:uid="{49EB169B-9D26-4956-990F-061D612A2D91}"/>
+    <hyperlink ref="A54" r:id="rId53" xr:uid="{102EBE77-E1CC-4DC6-8B91-223B46EE52D1}"/>
+    <hyperlink ref="A55" r:id="rId54" xr:uid="{CFBA3D75-5665-4423-A8A7-423E98FE08E6}"/>
+    <hyperlink ref="A56" r:id="rId55" xr:uid="{A57C4AE0-2FA2-4B88-BA9D-8B59F6D01F8B}"/>
+    <hyperlink ref="A57" r:id="rId56" xr:uid="{62DF92FC-0A00-4E33-B792-6C266DF58F0F}"/>
+    <hyperlink ref="A58" r:id="rId57" xr:uid="{F4FC44CF-BC7F-47C1-BC33-237507530E8D}"/>
+    <hyperlink ref="A59" r:id="rId58" xr:uid="{72E1774F-36AC-414A-BD4B-C6CBCF28F797}"/>
+    <hyperlink ref="A60" r:id="rId59" xr:uid="{B2C122A6-2BDF-4C40-A17C-F7264C374442}"/>
+    <hyperlink ref="A61" r:id="rId60" xr:uid="{DE4AF54F-F9D6-4881-87DA-0AD8B43FFB0D}"/>
+    <hyperlink ref="A62" r:id="rId61" xr:uid="{A9FE6BBE-54E7-441E-8CC9-FF0CF16D1492}"/>
+    <hyperlink ref="A63" r:id="rId62" xr:uid="{C158F021-37C1-4CD7-9D47-40A9F5F1F19C}"/>
+    <hyperlink ref="A64" r:id="rId63" xr:uid="{D1C27691-30F1-4985-AEB6-666C6BF546A1}"/>
+    <hyperlink ref="A65" r:id="rId64" xr:uid="{27703CEE-A444-4C59-9174-564E9780AB88}"/>
+    <hyperlink ref="A66" r:id="rId65" xr:uid="{4B5373A4-C972-430C-B28B-04F9548947CC}"/>
+    <hyperlink ref="A67" r:id="rId66" xr:uid="{6D20F7F4-9EEA-4B99-87C2-4F3F4C9A2CA7}"/>
+    <hyperlink ref="A68" r:id="rId67" xr:uid="{00D4B171-4273-4E1C-B30E-FD20D9474CA1}"/>
+    <hyperlink ref="A69" r:id="rId68" xr:uid="{36B5E2D7-2BD3-48EF-8726-146FACD70008}"/>
+    <hyperlink ref="A70" r:id="rId69" xr:uid="{663E41FF-CC8C-46F9-9D58-E279C50FA6E2}"/>
+    <hyperlink ref="A71" r:id="rId70" xr:uid="{01F41772-69B9-4C70-87FB-0A544A14D7B6}"/>
+    <hyperlink ref="A72" r:id="rId71" xr:uid="{81D0E439-90C6-489B-B776-C9FE01698AF0}"/>
+    <hyperlink ref="A73" r:id="rId72" xr:uid="{0ABD0DEB-B924-43F5-AF21-AD14DBF23AA8}"/>
+    <hyperlink ref="A74" r:id="rId73" xr:uid="{9F9332B3-3B8F-4E41-B6DD-F9A3E838F9C9}"/>
+    <hyperlink ref="A75" r:id="rId74" xr:uid="{3A5127E9-5D9B-43DD-A6A9-D478297FEAD6}"/>
+    <hyperlink ref="A76" r:id="rId75" xr:uid="{555802BD-0117-4C92-9484-1B5A079C9B77}"/>
+    <hyperlink ref="A77" r:id="rId76" xr:uid="{A1A231EE-0310-44CD-8177-7C2201E6103E}"/>
+    <hyperlink ref="A78" r:id="rId77" xr:uid="{BD00EFD5-E8D7-4F09-8052-2DDE26B57D85}"/>
+    <hyperlink ref="A79" r:id="rId78" xr:uid="{9226B8EE-4903-4F2B-B7FF-B1F3DF807632}"/>
+    <hyperlink ref="A80" r:id="rId79" xr:uid="{362DC7E3-9725-4CB8-98EE-80D1F8F1D991}"/>
+    <hyperlink ref="A81" r:id="rId80" xr:uid="{5E1AA0A0-1575-40A5-9089-ECD1AEF10907}"/>
+    <hyperlink ref="A82" r:id="rId81" xr:uid="{6CB63604-DB44-42FC-9557-0EF8F6AB36F8}"/>
+    <hyperlink ref="A83" r:id="rId82" xr:uid="{C815A4C4-7F95-4B66-ADD0-6571F648FCA7}"/>
+    <hyperlink ref="A84" r:id="rId83" xr:uid="{7B105B56-B6AD-45AE-A182-A7A036E4430B}"/>
+    <hyperlink ref="A85" r:id="rId84" xr:uid="{1C92D9FA-E47D-4134-954F-EE6090544912}"/>
+    <hyperlink ref="A86" r:id="rId85" xr:uid="{CB628E26-BE6D-4EC8-8926-CA3B4ED5470D}"/>
+    <hyperlink ref="A87" r:id="rId86" xr:uid="{850DC63F-7CA2-4C05-B904-C1AD82CDEC17}"/>
+    <hyperlink ref="A88" r:id="rId87" xr:uid="{159F22E2-F7B1-48F7-A6DE-39475025C1D9}"/>
+    <hyperlink ref="A89" r:id="rId88" xr:uid="{B5DE6F46-D0A0-41E1-865E-F9842CF86B6F}"/>
+    <hyperlink ref="A90" r:id="rId89" xr:uid="{E48E239E-A1F5-4631-9179-E853345BE5EA}"/>
+    <hyperlink ref="A91" r:id="rId90" xr:uid="{69D35F9E-B537-4B4C-95E9-7CA8E20D0A34}"/>
+    <hyperlink ref="A92" r:id="rId91" xr:uid="{3E6AC417-DF42-47B9-86E3-990A0FC69753}"/>
+    <hyperlink ref="A93" r:id="rId92" xr:uid="{28BD6162-A8CB-4332-9B06-148CBC143CC0}"/>
+    <hyperlink ref="A94" r:id="rId93" xr:uid="{0C76889A-45CC-45FE-AF11-192CC705D044}"/>
+    <hyperlink ref="A95" r:id="rId94" xr:uid="{4AFE48E1-6CB8-4250-A6DC-13B571C38B5E}"/>
+    <hyperlink ref="A96" r:id="rId95" xr:uid="{821D5588-3C8D-44AF-8E18-AB9C8D689E51}"/>
+    <hyperlink ref="A97" r:id="rId96" xr:uid="{7AF30CBC-6CD2-4058-8140-D18995F4EB0B}"/>
+    <hyperlink ref="A98" r:id="rId97" xr:uid="{CCADD1B7-705E-4E08-A4FF-5B77D3AFA4EC}"/>
+    <hyperlink ref="A99" r:id="rId98" xr:uid="{01767801-E612-4E82-9414-36F1FF21FAA3}"/>
+    <hyperlink ref="A100" r:id="rId99" xr:uid="{53758D03-4533-4FE7-9FEB-61A5C4C9D126}"/>
+    <hyperlink ref="A101" r:id="rId100" xr:uid="{D23D54C2-3D0C-4AAF-8D59-B67C49D1D9EB}"/>
+    <hyperlink ref="A102" r:id="rId101" xr:uid="{02DD77F6-B058-47AC-B04C-EA59687D8B5E}"/>
+    <hyperlink ref="A103" r:id="rId102" xr:uid="{087F95B1-20C2-417E-817B-6FBC64414488}"/>
+    <hyperlink ref="A104" r:id="rId103" xr:uid="{EE4D2143-8AEC-4FEF-95A2-7F8EE3A8A9E7}"/>
+    <hyperlink ref="A105" r:id="rId104" xr:uid="{566D74C0-F0A2-42FF-B42C-FA5C4CE6FD35}"/>
+    <hyperlink ref="A106" r:id="rId105" xr:uid="{51D49F65-5AB1-478E-BAC3-6AAA2B62E11E}"/>
+    <hyperlink ref="A107" r:id="rId106" xr:uid="{14B0B1CB-0028-4EDE-9745-0F2BACC9DF31}"/>
+    <hyperlink ref="A108" r:id="rId107" xr:uid="{93B8ADD2-9D01-4852-9BAE-B4762C659E21}"/>
+    <hyperlink ref="A109" r:id="rId108" xr:uid="{D2C0C028-7D23-49E3-A57E-2C4F9224C3EA}"/>
+    <hyperlink ref="A110" r:id="rId109" xr:uid="{08EEB716-A471-4C14-981F-53D46BDBD24A}"/>
+    <hyperlink ref="A111" r:id="rId110" xr:uid="{F5894C94-2F52-477F-A795-603875DFB535}"/>
+    <hyperlink ref="A112" r:id="rId111" xr:uid="{30AEBCCD-BB01-4EC6-9BD3-957A1B71EDDB}"/>
+    <hyperlink ref="A113" r:id="rId112" xr:uid="{FE816429-0B83-449A-B0B8-90D2856631BE}"/>
+    <hyperlink ref="A114" r:id="rId113" xr:uid="{5C7BF2AB-89BE-4AB4-814A-6F668F5C030D}"/>
+    <hyperlink ref="A115" r:id="rId114" xr:uid="{2B03AEB8-FD15-4B95-8CAC-6F4EC3B5D4FB}"/>
+    <hyperlink ref="A116" r:id="rId115" xr:uid="{AAA14CB3-3A45-4B2D-B2AF-FD44F4612F3C}"/>
+    <hyperlink ref="A117" r:id="rId116" xr:uid="{4973EED5-B603-4C2A-91BE-BB76C76BD594}"/>
+    <hyperlink ref="A118" r:id="rId117" xr:uid="{2281B3BA-D638-4B3B-A71B-CAD3E2385D75}"/>
+    <hyperlink ref="A119" r:id="rId118" xr:uid="{81144DF6-12CA-4B1C-BBAD-9A069F798936}"/>
+    <hyperlink ref="A120" r:id="rId119" xr:uid="{DC82C18F-57D7-45AA-9877-B2203592EFCD}"/>
+    <hyperlink ref="A121" r:id="rId120" xr:uid="{D3372687-F04D-4EBF-BB03-1FC0BA3244EC}"/>
+    <hyperlink ref="A122" r:id="rId121" xr:uid="{0EC333E2-29DA-4639-818A-848BB7D00712}"/>
+    <hyperlink ref="A123" r:id="rId122" xr:uid="{B50053E5-74B5-42CF-8A8F-5BB49F99C4BF}"/>
+    <hyperlink ref="A124" r:id="rId123" xr:uid="{5AB73072-C83E-4371-8DB8-C86D98CC14EB}"/>
+    <hyperlink ref="A125" r:id="rId124" xr:uid="{D34F7DBD-5576-4092-871B-1FD07A8EF7E1}"/>
+    <hyperlink ref="A126" r:id="rId125" xr:uid="{5FD3B3EE-60B4-4093-930C-06B694BBDB2D}"/>
+    <hyperlink ref="A127" r:id="rId126" xr:uid="{8B0027F9-97CE-4C66-A667-FCDFE07DF316}"/>
+    <hyperlink ref="A128" r:id="rId127" xr:uid="{1F562949-FA82-4141-9BF9-76318546F166}"/>
+    <hyperlink ref="A129" r:id="rId128" xr:uid="{1CA58188-00A7-4DFB-A91D-2806A09D2EDF}"/>
+    <hyperlink ref="A130" r:id="rId129" xr:uid="{E27DD09D-41D1-49F7-B55B-2591351E3EC6}"/>
+    <hyperlink ref="A131" r:id="rId130" xr:uid="{F8AB7CE2-76BD-4B81-A628-8D6A1FCAA5B0}"/>
+    <hyperlink ref="A132" r:id="rId131" xr:uid="{D86D4458-F227-47F8-8114-3822A75539AB}"/>
+    <hyperlink ref="A133" r:id="rId132" xr:uid="{08E2EA5A-20FC-4528-A0B4-C9D92E4E4419}"/>
+    <hyperlink ref="A134" r:id="rId133" xr:uid="{6D7F1D04-7326-4569-9A42-96A3E61301DE}"/>
+    <hyperlink ref="A135" r:id="rId134" xr:uid="{F022B027-5656-4733-9595-FE1FBDC7FBCA}"/>
+    <hyperlink ref="A136" r:id="rId135" xr:uid="{58E572CD-BDE0-4D0A-AAF3-F09A7B3CDF42}"/>
+    <hyperlink ref="A137" r:id="rId136" xr:uid="{AE7DDDDF-5730-4453-97B9-96C9799962E1}"/>
+    <hyperlink ref="A138" r:id="rId137" xr:uid="{F03BDAE5-FE2A-40F6-A24E-C3928B10768F}"/>
+    <hyperlink ref="A139" r:id="rId138" xr:uid="{0180557C-3C97-4E2B-93C0-C97A05D76AE7}"/>
+    <hyperlink ref="A140" r:id="rId139" xr:uid="{7C9BB6D5-70C1-43E0-8709-82D61CB9CF41}"/>
+    <hyperlink ref="A141" r:id="rId140" xr:uid="{60B848AA-0D02-402A-A0B2-A18C5EA5723A}"/>
+    <hyperlink ref="A142" r:id="rId141" xr:uid="{5638AF2A-A356-4083-B002-2EF28F4C4CCF}"/>
+    <hyperlink ref="A143" r:id="rId142" xr:uid="{D43CE2EB-7062-40EA-86A5-E7EE78D3ED07}"/>
+    <hyperlink ref="A144" r:id="rId143" xr:uid="{F7D9D8CC-5BA9-4687-B978-917648533134}"/>
+    <hyperlink ref="A145" r:id="rId144" xr:uid="{5D6466F5-4A46-4EBD-BF97-9FCB7C00AD53}"/>
+    <hyperlink ref="A146" r:id="rId145" xr:uid="{161513BE-EF61-4DA9-9E5A-B6A4F2A9EDF1}"/>
+    <hyperlink ref="A147" r:id="rId146" xr:uid="{FFAB3EFC-C334-4B2B-AE54-0CA53E3F8BA7}"/>
+    <hyperlink ref="A148" r:id="rId147" xr:uid="{CF862C4F-A4CB-4707-9F88-B87E70EF3B5E}"/>
+    <hyperlink ref="A149" r:id="rId148" xr:uid="{C175A8DC-8C9A-40A3-A3D1-93818B477422}"/>
+    <hyperlink ref="A150" r:id="rId149" xr:uid="{168E6B34-C097-40F3-9378-7B5FB01535F7}"/>
+    <hyperlink ref="A151" r:id="rId150" xr:uid="{C679535D-F4A6-4ED2-8C40-10EA9D8AB2FD}"/>
+    <hyperlink ref="A152" r:id="rId151" xr:uid="{2866E4CC-3DC7-4A13-849A-09F031B085EF}"/>
+    <hyperlink ref="A153" r:id="rId152" xr:uid="{0851C9AF-47AE-4619-B150-C2FFEDDF8808}"/>
+    <hyperlink ref="A154" r:id="rId153" xr:uid="{7C928AD8-D2EC-48D0-A5E8-5D3A09049CE1}"/>
+    <hyperlink ref="A155" r:id="rId154" xr:uid="{14CE17BB-AD15-4736-AC38-E53A5F48D51A}"/>
+    <hyperlink ref="A156" r:id="rId155" xr:uid="{A8C957AA-AC04-4D7A-BE21-0966554E2173}"/>
+    <hyperlink ref="A157" r:id="rId156" xr:uid="{4030FC7B-D9B9-4DD6-A913-F1CC98AF9148}"/>
+    <hyperlink ref="A158" r:id="rId157" xr:uid="{4BDAB404-7EC0-4B40-A946-65B8B9CD4A12}"/>
+    <hyperlink ref="A159" r:id="rId158" xr:uid="{41B2B442-1824-40BD-8E5C-B196975FF1FD}"/>
+    <hyperlink ref="A160" r:id="rId159" xr:uid="{94550EE4-EC03-42AE-ABF3-3F9657295E7F}"/>
+    <hyperlink ref="A161" r:id="rId160" xr:uid="{16EBE022-F854-4D69-9EC6-5E5E65A23B72}"/>
+    <hyperlink ref="A162" r:id="rId161" xr:uid="{108893B3-3695-48D4-8E21-F0C492E61F3C}"/>
+    <hyperlink ref="A163" r:id="rId162" xr:uid="{481BF149-AD83-48D4-9E26-E669DBCB195C}"/>
+    <hyperlink ref="A164" r:id="rId163" xr:uid="{C8076BC9-8D0A-4CB1-A6E8-1C40DD07258E}"/>
+    <hyperlink ref="A165" r:id="rId164" xr:uid="{64FEBDEF-C894-4F12-AE41-611FB581DB66}"/>
+    <hyperlink ref="A166" r:id="rId165" xr:uid="{06AFDEF4-7D35-43D7-AC75-52714B5DC600}"/>
+    <hyperlink ref="A167" r:id="rId166" xr:uid="{A7C5F366-2DB0-4A9F-936D-D005502E4095}"/>
+    <hyperlink ref="A168" r:id="rId167" xr:uid="{BB3C43C5-7089-4626-A51E-908B07B0ACE7}"/>
+    <hyperlink ref="A169" r:id="rId168" xr:uid="{A42AE297-1EAF-4830-8100-03D628CA59DF}"/>
+    <hyperlink ref="A170" r:id="rId169" xr:uid="{C2E5B80F-45B6-4DC6-B819-407B877A6F10}"/>
+    <hyperlink ref="A171" r:id="rId170" xr:uid="{DFB42FAB-AA7C-447C-8D80-5EFF4CA4A2B6}"/>
+    <hyperlink ref="A172" r:id="rId171" xr:uid="{FD0F318F-E01C-4358-B7D0-F7F9BF6E76A1}"/>
+    <hyperlink ref="A173" r:id="rId172" xr:uid="{8ABE2496-5E9F-44F4-ACA3-7B2FAFCBE46C}"/>
+    <hyperlink ref="A174" r:id="rId173" xr:uid="{9EB5EB72-2163-476B-A1A6-050C1F8EB956}"/>
+    <hyperlink ref="A175" r:id="rId174" xr:uid="{A12A80C1-3301-43AF-A0A3-5440C2F50EE5}"/>
+    <hyperlink ref="A176" r:id="rId175" xr:uid="{E64E94FE-B7F0-4FB7-BF56-FD9B84195E3C}"/>
+    <hyperlink ref="A177" r:id="rId176" xr:uid="{EC0EC532-0A28-4E8F-9207-C42F1150E936}"/>
+    <hyperlink ref="A178" r:id="rId177" xr:uid="{D0C27CC1-A7BA-461E-9CDB-94E1B95365A4}"/>
+    <hyperlink ref="A179" r:id="rId178" xr:uid="{B7BA84F4-DB11-4C8E-BCA3-E916CFCCC970}"/>
+    <hyperlink ref="A180" r:id="rId179" xr:uid="{1AE20649-BC85-4546-A7E3-ABCE3E12E2E7}"/>
+    <hyperlink ref="A181" r:id="rId180" xr:uid="{4EF15FC1-7D63-48BC-AF73-49DB93105782}"/>
+    <hyperlink ref="A182" r:id="rId181" xr:uid="{458D1A30-A57F-42F4-86FA-0450D72568DF}"/>
+    <hyperlink ref="A183" r:id="rId182" xr:uid="{69EC23C6-A651-42A6-8BBC-0A075B2F324A}"/>
+    <hyperlink ref="A184" r:id="rId183" xr:uid="{1F7EA4F8-C121-493C-AAFF-C9C272F92AD5}"/>
+    <hyperlink ref="A185" r:id="rId184" xr:uid="{3D6E2A34-A65D-44FD-AFDE-F6DA8D58C46D}"/>
+    <hyperlink ref="A186" r:id="rId185" xr:uid="{8A08A1A7-64BA-48B0-94AE-E828918FBB4C}"/>
+    <hyperlink ref="A187" r:id="rId186" xr:uid="{CC15C183-2ED8-4074-8F6A-CAFBEBCA095A}"/>
+    <hyperlink ref="A188" r:id="rId187" xr:uid="{A6B39A3F-2D74-46AE-B949-F534D5357392}"/>
+    <hyperlink ref="A189" r:id="rId188" xr:uid="{BF849EA7-4BA9-4C85-B7B6-DD16583DEA44}"/>
+    <hyperlink ref="A190" r:id="rId189" xr:uid="{C7CE2052-5BE0-4E0D-B5F2-FC0236F65341}"/>
+    <hyperlink ref="A191" r:id="rId190" xr:uid="{1EAE00B8-6A19-4EEA-B04D-BAB7413A3FEF}"/>
+    <hyperlink ref="A192" r:id="rId191" xr:uid="{04E22AC3-271D-4D2E-B7FE-8CBD1B8DEDAC}"/>
+    <hyperlink ref="A193" r:id="rId192" xr:uid="{0F0B6D4E-8F7E-4FEC-8BC7-0FD9EA982393}"/>
+    <hyperlink ref="A194" r:id="rId193" xr:uid="{5CFD6912-C272-4C97-91DE-AF088DA1C3CF}"/>
+    <hyperlink ref="A195" r:id="rId194" xr:uid="{509F940A-1B33-4B42-9FFC-949CF9F44B66}"/>
+    <hyperlink ref="A196" r:id="rId195" xr:uid="{FF5A075F-3354-479C-BFD2-DFBF20EBE154}"/>
+    <hyperlink ref="A197" r:id="rId196" xr:uid="{872E6195-31E7-47D2-9F7C-5FDDCEFE8700}"/>
+    <hyperlink ref="A198" r:id="rId197" xr:uid="{A72DA58A-A0B5-411C-81C5-26930CF3A664}"/>
+    <hyperlink ref="A199" r:id="rId198" xr:uid="{9C9E207E-1A85-4DC3-8C97-41C68A73039A}"/>
+    <hyperlink ref="A200" r:id="rId199" xr:uid="{D787D663-8C48-43D5-B29D-15F9140B8F05}"/>
+    <hyperlink ref="A201" r:id="rId200" xr:uid="{F14FDE22-CE79-45FD-8457-CD65F0A9AC19}"/>
+    <hyperlink ref="A202" r:id="rId201" xr:uid="{597BFD59-6A55-4C5F-9631-06491A4157DF}"/>
+    <hyperlink ref="A203" r:id="rId202" xr:uid="{75EE9C16-28F3-4992-A1A4-8B744872356C}"/>
+    <hyperlink ref="A204" r:id="rId203" xr:uid="{48206D6C-427B-4FC6-B194-3CF3574DFAB3}"/>
+    <hyperlink ref="A205" r:id="rId204" xr:uid="{DC96E1CF-582C-4E7D-80D8-85871436AB19}"/>
+    <hyperlink ref="A206" r:id="rId205" xr:uid="{906AA231-F7CE-43E0-9AE1-53C18D273D24}"/>
+    <hyperlink ref="A207" r:id="rId206" xr:uid="{90C21C1A-9270-41C4-8EA9-36EB39563437}"/>
+    <hyperlink ref="A208" r:id="rId207" xr:uid="{12507AB8-C666-40CA-AA92-49ED06A24C46}"/>
+    <hyperlink ref="A209" r:id="rId208" xr:uid="{4DF18A57-AC6C-4598-BB1D-F976DC0CBBCD}"/>
+    <hyperlink ref="A210" r:id="rId209" xr:uid="{3278FEE5-4DB8-4242-8C9B-F05B3DA30962}"/>
+    <hyperlink ref="A211" r:id="rId210" xr:uid="{FBE3C03E-D33C-4AC9-9B5D-C93F7C2BEB04}"/>
+    <hyperlink ref="A212" r:id="rId211" xr:uid="{6C0D00F9-1B53-443C-BB04-5B7EEF2FC290}"/>
+    <hyperlink ref="A213" r:id="rId212" xr:uid="{F206BBD1-71AD-40C5-8323-BCCC56F58E36}"/>
+    <hyperlink ref="A214" r:id="rId213" xr:uid="{83972FDF-FC22-420B-B5F0-6409196B4293}"/>
+    <hyperlink ref="A215" r:id="rId214" xr:uid="{345818F5-4C96-4174-B5D9-901E65B79659}"/>
+    <hyperlink ref="A216" r:id="rId215" xr:uid="{FC5DB154-AC54-44B7-932C-3B2C3E6F93C7}"/>
+    <hyperlink ref="A217" r:id="rId216" xr:uid="{136155C9-4248-4569-BA94-9DDBB8515576}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>

</xml_diff>